<commit_message>
fix: track only unique person imports by checking existence before incrementing counter
</commit_message>
<xml_diff>
--- a/bani muzakki 2.xlsx
+++ b/bani muzakki 2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4dd770f5288dd514/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4dd770f5288dd514/Documents/GitHub/familyhood.my.id/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{870BD3E6-2C3D-4F2D-9816-F863933228ED}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB80F8E-BB6F-464C-9455-26EC13A679BF}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{AF1F46D2-AE81-41B2-8BCC-10330EF8BD9C}">
+    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{AF1F46D2-AE81-41B2-8BCC-10330EF8BD9C}">
       <text>
         <r>
           <rPr>
@@ -56,7 +56,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{C99F29C0-970A-46FD-88BD-45AA74722360}">
+    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{C99F29C0-970A-46FD-88BD-45AA74722360}">
       <text>
         <r>
           <rPr>
@@ -68,7 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{845CB564-AED8-4E26-A41F-687C241CAEB5}">
+    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{845CB564-AED8-4E26-A41F-687C241CAEB5}">
       <text>
         <r>
           <rPr>
@@ -80,7 +80,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{E4BCF476-780D-452E-8F0F-E0E8B44286C5}">
+    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{E4BCF476-780D-452E-8F0F-E0E8B44286C5}">
       <text>
         <r>
           <rPr>
@@ -92,7 +92,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{2BA95F4A-7354-4FDC-80BD-2133092C102B}">
+    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{2BA95F4A-7354-4FDC-80BD-2133092C102B}">
       <text>
         <r>
           <rPr>
@@ -104,7 +104,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D79" authorId="0" shapeId="0" xr:uid="{462043AC-24E8-4B01-BF3B-DBCE99D58342}">
+    <comment ref="D80" authorId="0" shapeId="0" xr:uid="{462043AC-24E8-4B01-BF3B-DBCE99D58342}">
       <text>
         <r>
           <rPr>
@@ -116,7 +116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C81" authorId="0" shapeId="0" xr:uid="{FB1C37D4-72C2-4D9F-A3A1-BE7E0FCFA979}">
+    <comment ref="C82" authorId="0" shapeId="0" xr:uid="{FB1C37D4-72C2-4D9F-A3A1-BE7E0FCFA979}">
       <text>
         <r>
           <rPr>
@@ -128,7 +128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D101" authorId="0" shapeId="0" xr:uid="{B95DBADC-5274-4970-B2EF-BA6EDE495B32}">
+    <comment ref="D102" authorId="0" shapeId="0" xr:uid="{B95DBADC-5274-4970-B2EF-BA6EDE495B32}">
       <text>
         <r>
           <rPr>
@@ -140,7 +140,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D109" authorId="0" shapeId="0" xr:uid="{3D1FECAA-E9AC-469D-968C-B08407A7E555}">
+    <comment ref="D110" authorId="0" shapeId="0" xr:uid="{3D1FECAA-E9AC-469D-968C-B08407A7E555}">
       <text>
         <r>
           <rPr>
@@ -152,7 +152,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D126" authorId="0" shapeId="0" xr:uid="{652EA41B-5E8F-4E35-965E-DC62524B30E4}">
+    <comment ref="D127" authorId="0" shapeId="0" xr:uid="{652EA41B-5E8F-4E35-965E-DC62524B30E4}">
       <text>
         <r>
           <rPr>
@@ -164,7 +164,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D131" authorId="0" shapeId="0" xr:uid="{EB3699E2-FEF4-456B-8D80-19A0E1F73915}">
+    <comment ref="D132" authorId="0" shapeId="0" xr:uid="{EB3699E2-FEF4-456B-8D80-19A0E1F73915}">
       <text>
         <r>
           <rPr>
@@ -177,7 +177,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E134" authorId="0" shapeId="0" xr:uid="{248F1982-A68D-4075-B49E-DFE7A3EEE35C}">
+    <comment ref="E135" authorId="0" shapeId="0" xr:uid="{248F1982-A68D-4075-B49E-DFE7A3EEE35C}">
       <text>
         <r>
           <rPr>
@@ -190,7 +190,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D136" authorId="0" shapeId="0" xr:uid="{146CA70A-EBE9-449B-8DB8-250759CFD077}">
+    <comment ref="D137" authorId="0" shapeId="0" xr:uid="{146CA70A-EBE9-449B-8DB8-250759CFD077}">
       <text>
         <r>
           <rPr>
@@ -203,7 +203,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D153" authorId="0" shapeId="0" xr:uid="{F773B15B-9F7C-43C0-94D6-9AFFA8926436}">
+    <comment ref="D154" authorId="0" shapeId="0" xr:uid="{F773B15B-9F7C-43C0-94D6-9AFFA8926436}">
       <text>
         <r>
           <rPr>
@@ -215,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E170" authorId="0" shapeId="0" xr:uid="{EF3CCB78-BD13-4482-8109-9AB59DD642A1}">
+    <comment ref="E171" authorId="0" shapeId="0" xr:uid="{EF3CCB78-BD13-4482-8109-9AB59DD642A1}">
       <text>
         <r>
           <rPr>
@@ -227,7 +227,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C179" authorId="0" shapeId="0" xr:uid="{5BDAADBF-92C0-4462-823A-597F00B6DA8B}">
+    <comment ref="C180" authorId="0" shapeId="0" xr:uid="{5BDAADBF-92C0-4462-823A-597F00B6DA8B}">
       <text>
         <r>
           <rPr>
@@ -239,7 +239,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C183" authorId="0" shapeId="0" xr:uid="{7115E3C1-ADBA-429A-AB3C-37FAE8BAC9C7}">
+    <comment ref="C184" authorId="0" shapeId="0" xr:uid="{7115E3C1-ADBA-429A-AB3C-37FAE8BAC9C7}">
       <text>
         <r>
           <rPr>
@@ -251,7 +251,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E230" authorId="0" shapeId="0" xr:uid="{EEE70887-3507-410D-908B-63439A987A79}">
+    <comment ref="E231" authorId="0" shapeId="0" xr:uid="{EEE70887-3507-410D-908B-63439A987A79}">
       <text>
         <r>
           <rPr>
@@ -264,7 +264,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D293" authorId="0" shapeId="0" xr:uid="{66A4E9CF-C1FD-417D-8D92-41FDF2D33936}">
+    <comment ref="D294" authorId="0" shapeId="0" xr:uid="{66A4E9CF-C1FD-417D-8D92-41FDF2D33936}">
       <text>
         <r>
           <rPr>
@@ -276,7 +276,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D315" authorId="0" shapeId="0" xr:uid="{F8960E51-4F3B-4B2F-AE76-558F4A32BC38}">
+    <comment ref="D316" authorId="0" shapeId="0" xr:uid="{F8960E51-4F3B-4B2F-AE76-558F4A32BC38}">
       <text>
         <r>
           <rPr>
@@ -293,7 +293,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="328">
   <si>
     <t>MUZAKKI + ZAKIYAH</t>
   </si>
@@ -1253,13 +1253,37 @@
   </si>
   <si>
     <t>SABIQ ZAIN MAKARIM</t>
+  </si>
+  <si>
+    <t>Generasi 1</t>
+  </si>
+  <si>
+    <t>Generasi 2</t>
+  </si>
+  <si>
+    <t>Generasi 3</t>
+  </si>
+  <si>
+    <t>Generasi 4</t>
+  </si>
+  <si>
+    <t>Generasi 5</t>
+  </si>
+  <si>
+    <t>Generasi 6</t>
+  </si>
+  <si>
+    <t>Generasi 7</t>
+  </si>
+  <si>
+    <t>Generasi 8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1273,13 +1297,25 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE5E7EB"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1294,8 +1330,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1611,1613 +1648,1648 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C629E1E-B955-4A3C-B56E-5C952373FF63}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F320"/>
+  <dimension ref="A1:H362"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="6" width="4.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="56.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C3" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E11" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E12" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D13" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E14" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E15" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D16" t="s">
+    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E17" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="18" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C19" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
+    <row r="22" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E22" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="23" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D27" t="s">
+    <row r="28" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E28" t="s">
+    <row r="29" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="F29" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="30" spans="3:6" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E31" t="s">
+    <row r="32" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="F32" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="33" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E35" t="s">
+    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D36" t="s">
+    <row r="37" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D37" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E37" t="s">
+    <row r="38" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F38" t="s">
+    <row r="39" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E39" t="s">
+    <row r="40" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E40" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D40" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="41" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E42" t="s">
+    <row r="43" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D43" t="s">
+    <row r="44" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D44" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E44" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="45" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E50" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D50" t="s">
+    <row r="51" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D51" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E51" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="52" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E53" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D53" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D55" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E55" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="56" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E57" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D57" t="s">
+    <row r="58" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D58" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C58" t="s">
+    <row r="59" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D59" t="s">
+    <row r="60" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D60" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E60" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="61" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="64" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E64" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D64" t="s">
+    <row r="65" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D65" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="65" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E65" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="66" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="67" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="68" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="69" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E69" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D69" t="s">
+    <row r="70" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D70" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C70" t="s">
+    <row r="71" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C71" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D71" t="s">
+    <row r="72" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D72" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="72" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E72" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="73" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="74" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="75" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E75" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D75" t="s">
+    <row r="76" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D76" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="76" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E76" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="77" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="79" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E79" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D79" t="s">
+    <row r="80" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D80" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E80" t="s">
+    <row r="81" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E81" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
+    <row r="82" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="82" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D82" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="83" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="84" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D84" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E84" t="s">
+    <row r="85" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E85" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D85" t="s">
+    <row r="86" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D86" t="s">
         <v>84</v>
-      </c>
-    </row>
-    <row r="86" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C86" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="87" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="88" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="89" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C89" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D89" t="s">
+    <row r="90" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D90" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E90" t="s">
+    <row r="91" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E91" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="91" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D91" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="92" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="93" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D93" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D94" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row r="94" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C94" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="95" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="96" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C96" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D96" t="s">
+    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D97" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E97" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E98" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="99" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="E99" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D99" t="s">
+    <row r="100" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D100" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E100" t="s">
+    <row r="101" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="E101" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="101" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D101" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="104" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D104" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B104" t="s">
+    <row r="105" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C105" t="s">
+    <row r="106" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C106" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D106" t="s">
+    <row r="107" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D107" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="107" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E107" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="109" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="E109" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D109" t="s">
+    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D110" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E110" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E112" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E113" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="114" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E114" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D114" t="s">
+    <row r="115" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D115" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="115" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E115" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="116" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="117" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="118" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E118" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="119" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E119" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D119" t="s">
+    <row r="120" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D120" t="s">
         <v>118</v>
-      </c>
-    </row>
-    <row r="120" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E120" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="121" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E121" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="122" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E122" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D122" t="s">
+    <row r="123" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D123" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="123" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E123" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="124" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="125" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E125" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C125" t="s">
+    <row r="126" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C126" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D126" t="s">
+    <row r="127" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D127" t="s">
         <v>125</v>
-      </c>
-    </row>
-    <row r="127" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E127" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="128" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E128" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="129" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E129" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D129" t="s">
+    <row r="130" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D130" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="130" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E130" t="s">
+    <row r="131" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E131" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="131" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D131" t="s">
+    <row r="132" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D132" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="132" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E132" t="s">
+    <row r="133" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E133" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="133" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D133" t="s">
+    <row r="134" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D134" t="s">
         <v>132</v>
-      </c>
-    </row>
-    <row r="134" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E134" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="135" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E135" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="136" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E136" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="136" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D136" t="s">
+    <row r="137" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D137" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="137" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E137" t="s">
+    <row r="138" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E138" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="138" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D138" t="s">
+    <row r="139" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D139" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="139" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E139" t="s">
+    <row r="140" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E140" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="140" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C140" t="s">
+    <row r="141" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C141" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="141" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D141" t="s">
+    <row r="142" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D142" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="142" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E142" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="143" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E143" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="144" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E144" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="144" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D144" t="s">
+    <row r="145" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D145" t="s">
         <v>143</v>
-      </c>
-    </row>
-    <row r="145" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E145" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="146" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E146" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="147" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E147" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="147" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C147" t="s">
+    <row r="148" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C148" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="148" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D148" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="149" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D149" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="150" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D150" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E150" t="s">
+    <row r="151" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E151" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="151" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D151" t="s">
+    <row r="152" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D152" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="152" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C152" t="s">
+    <row r="153" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C153" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="153" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D153" t="s">
+    <row r="154" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D154" t="s">
         <v>152</v>
-      </c>
-    </row>
-    <row r="154" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E154" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="155" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E155" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="156" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E156" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="156" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D156" t="s">
+    <row r="157" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D157" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="157" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C157" t="s">
+    <row r="158" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C158" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="158" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D158" t="s">
+    <row r="159" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D159" t="s">
         <v>157</v>
-      </c>
-    </row>
-    <row r="159" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E159" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="160" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E160" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="161" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E161" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="161" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D161" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="162" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D162" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="163" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D163" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="163" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C163" t="s">
+    <row r="164" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C164" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="164" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D164" t="s">
+    <row r="165" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D165" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="165" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E165" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="166" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="167" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E167" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="168" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E168" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="169" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E169" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="169" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D169" t="s">
+    <row r="170" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D170" t="s">
         <v>168</v>
-      </c>
-    </row>
-    <row r="170" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E170" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="171" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E171" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="172" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E172" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="173" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E173" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="174" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E174" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="175" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E175" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="176" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E176" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="176" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D176" t="s">
+    <row r="177" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D177" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="177" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E177" t="s">
+    <row r="178" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E178" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="178" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D178" t="s">
+    <row r="179" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D179" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="179" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C179" t="s">
+    <row r="180" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C180" t="s">
         <v>178</v>
-      </c>
-    </row>
-    <row r="180" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D180" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="181" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D181" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="182" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D182" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="183" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D183" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="183" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C183" t="s">
+    <row r="184" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C184" t="s">
         <v>182</v>
-      </c>
-    </row>
-    <row r="184" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D184" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="185" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D185" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="186" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D186" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="187" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D187" t="s">
         <v>185</v>
-      </c>
-    </row>
-    <row r="187" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C187" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="188" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C188" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="189" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C189" t="s">
         <v>187</v>
-      </c>
-    </row>
-    <row r="189" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D189" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="190" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D190" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="191" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D191" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="191" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E191" t="s">
+    <row r="192" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E192" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="192" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D192" t="s">
+    <row r="193" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D193" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="193" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E193" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="194" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E194" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="195" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E195" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="196" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E196" t="s">
         <v>194</v>
-      </c>
-    </row>
-    <row r="196" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D196" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="197" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D197" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="198" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D198" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="199" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D199" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="199" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C199" t="s">
+    <row r="200" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C200" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="200" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B200" t="s">
+    <row r="201" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B201" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="201" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C201" t="s">
+    <row r="202" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C202" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="202" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D202" t="s">
+    <row r="203" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D203" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="203" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E203" t="s">
+    <row r="204" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E204" t="s">
         <v>202</v>
-      </c>
-    </row>
-    <row r="204" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="F204" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="205" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F205" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="206" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F206" t="s">
         <v>204</v>
-      </c>
-    </row>
-    <row r="206" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E206" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="207" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E207" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="208" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E208" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="208" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D208" t="s">
+    <row r="209" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D209" t="s">
         <v>207</v>
-      </c>
-    </row>
-    <row r="209" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E209" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="210" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E210" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="211" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E211" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="212" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E212" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="213" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E213" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="214" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E214" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="215" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E215" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="215" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D215" t="s">
+    <row r="216" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D216" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="216" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E216" t="s">
+    <row r="217" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E217" t="s">
         <v>215</v>
-      </c>
-    </row>
-    <row r="217" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F217" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="218" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F218" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="219" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F219" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="220" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="F220" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="220" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E220" t="s">
+    <row r="221" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E221" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="221" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F221" t="s">
+    <row r="222" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="F222" t="s">
         <v>220</v>
-      </c>
-    </row>
-    <row r="222" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E222" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="223" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E223" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="224" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E224" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="225" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E225" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="226" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E226" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="227" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E227" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="227" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D227" t="s">
+    <row r="228" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D228" t="s">
         <v>226</v>
-      </c>
-    </row>
-    <row r="228" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E228" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="229" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E229" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="230" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E230" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="231" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E231" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="232" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E232" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="233" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E233" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="233" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D233" t="s">
+    <row r="234" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D234" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="234" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E234" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="235" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E235" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="236" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E236" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="236" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D236" t="s">
+    <row r="237" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D237" t="s">
         <v>235</v>
-      </c>
-    </row>
-    <row r="237" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E237" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="238" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E238" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="239" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="E239" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="239" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D239" t="s">
+    <row r="240" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D240" t="s">
         <v>238</v>
-      </c>
-    </row>
-    <row r="240" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E240" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="241" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E241" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="242" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E242" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="243" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E243" t="s">
         <v>241</v>
-      </c>
-    </row>
-    <row r="243" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C243" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="244" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C244" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="245" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C245" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="245" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D245" t="s">
+    <row r="246" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D246" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="246" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E246" t="s">
+    <row r="247" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E247" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="247" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D247" t="s">
+    <row r="248" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D248" t="s">
         <v>246</v>
-      </c>
-    </row>
-    <row r="248" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E248" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="249" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E249" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="250" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E250" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="251" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E251" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="251" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D251" t="s">
+    <row r="252" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D252" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="252" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E252" t="s">
+    <row r="253" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E253" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="253" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D253" t="s">
+    <row r="254" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D254" t="s">
         <v>252</v>
-      </c>
-    </row>
-    <row r="254" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E254" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="255" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E255" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="256" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E256" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="256" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D256" t="s">
+    <row r="257" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D257" t="s">
         <v>255</v>
-      </c>
-    </row>
-    <row r="257" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E257" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="258" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E258" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="259" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E259" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="260" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E260" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="260" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C260" t="s">
+    <row r="261" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C261" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="261" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D261" t="s">
+    <row r="262" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D262" t="s">
         <v>260</v>
-      </c>
-    </row>
-    <row r="262" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E262" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="263" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E263" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="264" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E264" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="265" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E265" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="266" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E266" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="266" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D266" t="s">
+    <row r="267" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D267" t="s">
         <v>265</v>
-      </c>
-    </row>
-    <row r="267" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E267" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="268" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E268" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="269" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E269" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="270" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E270" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="270" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D270" t="s">
+    <row r="271" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D271" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="271" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C271" t="s">
+    <row r="272" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C272" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="272" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D272" t="s">
+    <row r="273" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D273" t="s">
         <v>271</v>
-      </c>
-    </row>
-    <row r="273" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E273" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="274" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E274" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="275" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E275" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="276" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E276" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="276" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D276" t="s">
+    <row r="277" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D277" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="277" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E277" t="s">
+    <row r="278" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E278" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="278" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D278" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="279" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D279" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="280" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D280" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="280" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C280" t="s">
+    <row r="281" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C281" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="281" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D281" t="s">
+    <row r="282" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D282" t="s">
         <v>280</v>
-      </c>
-    </row>
-    <row r="282" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E282" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="283" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E283" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="284" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E284" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="285" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E285" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="285" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D285" t="s">
+    <row r="286" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D286" t="s">
         <v>284</v>
-      </c>
-    </row>
-    <row r="286" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E286" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="287" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E287" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="288" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E288" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="289" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E289" t="s">
         <v>287</v>
-      </c>
-    </row>
-    <row r="289" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D289" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="290" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D290" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="291" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D291" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="291" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E291" t="s">
+    <row r="292" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E292" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="292" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C292" t="s">
+    <row r="293" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C293" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="293" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D293" t="s">
+    <row r="294" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D294" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="294" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C294" t="s">
+    <row r="295" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C295" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="295" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D295" t="s">
+    <row r="296" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D296" t="s">
         <v>294</v>
-      </c>
-    </row>
-    <row r="296" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E296" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="297" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E297" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="298" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E298" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="299" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E299" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="299" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D299" t="s">
+    <row r="300" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D300" t="s">
         <v>298</v>
-      </c>
-    </row>
-    <row r="300" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E300" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="301" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E301" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="302" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E302" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="303" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E303" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="303" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D303" t="s">
+    <row r="304" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D304" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="304" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E304" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="305" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E305" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="306" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E306" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="307" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E307" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="308" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E308" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="309" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E309" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="309" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D309" t="s">
+    <row r="310" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D310" t="s">
         <v>308</v>
-      </c>
-    </row>
-    <row r="310" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E310" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="311" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E311" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="312" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E312" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="313" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E313" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="313" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D313" t="s">
+    <row r="314" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D314" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="314" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C314" t="s">
+    <row r="315" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C315" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="315" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D315" t="s">
+    <row r="316" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="D316" t="s">
         <v>314</v>
-      </c>
-    </row>
-    <row r="316" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C316" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="317" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C317" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="318" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C318" t="s">
         <v>316</v>
-      </c>
-    </row>
-    <row r="318" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D318" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="319" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D319" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="320" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D320" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="321" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D321" t="s">
         <v>319</v>
+      </c>
+    </row>
+    <row r="362" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F362">
+        <f>COUNTA(F2:F361)</f>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Please provide the file changes or a summary of the modifications you made so I can generate the commit message for you.
</commit_message>
<xml_diff>
--- a/bani muzakki 2.xlsx
+++ b/bani muzakki 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4dd770f5288dd514/Documents/GitHub/familyhood.my.id/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{870BD3E6-2C3D-4F2D-9816-F863933228ED}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1786E367-F2F0-4A54-A4C7-2C9C66DF4E48}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB80F8E-BB6F-464C-9455-26EC13A679BF}"/>
   </bookViews>
@@ -293,7 +293,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="326">
   <si>
     <t>MUZAKKI + ZAKIYAH</t>
   </si>
@@ -1271,12 +1271,6 @@
   </si>
   <si>
     <t>Generasi 6</t>
-  </si>
-  <si>
-    <t>Generasi 7</t>
-  </si>
-  <si>
-    <t>Generasi 8</t>
   </si>
 </sst>
 </file>
@@ -1348,6 +1342,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1648,7 +1646,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C629E1E-B955-4A3C-B56E-5C952373FF63}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H362"/>
+  <dimension ref="A1:F362"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -1657,10 +1655,9 @@
     <col min="4" max="4" width="67" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="56.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>320</v>
       </c>
@@ -1679,84 +1676,78 @@
       <c r="F1" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
feat: add Level Line tree visualization view and include new Excel file
</commit_message>
<xml_diff>
--- a/bani muzakki 2.xlsx
+++ b/bani muzakki 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4dd770f5288dd514/Documents/GitHub/familyhood.my.id/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1786E367-F2F0-4A54-A4C7-2C9C66DF4E48}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D12EDC8A-B394-43F1-91E2-CF16B48B558C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB80F8E-BB6F-464C-9455-26EC13A679BF}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{AF1F46D2-AE81-41B2-8BCC-10330EF8BD9C}">
+    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{AF1F46D2-AE81-41B2-8BCC-10330EF8BD9C}">
       <text>
         <r>
           <rPr>
@@ -56,7 +56,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{C99F29C0-970A-46FD-88BD-45AA74722360}">
+    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{C99F29C0-970A-46FD-88BD-45AA74722360}">
       <text>
         <r>
           <rPr>
@@ -68,7 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{845CB564-AED8-4E26-A41F-687C241CAEB5}">
+    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{845CB564-AED8-4E26-A41F-687C241CAEB5}">
       <text>
         <r>
           <rPr>
@@ -80,7 +80,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{E4BCF476-780D-452E-8F0F-E0E8B44286C5}">
+    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{E4BCF476-780D-452E-8F0F-E0E8B44286C5}">
       <text>
         <r>
           <rPr>
@@ -92,7 +92,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{2BA95F4A-7354-4FDC-80BD-2133092C102B}">
+    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{2BA95F4A-7354-4FDC-80BD-2133092C102B}">
       <text>
         <r>
           <rPr>
@@ -104,7 +104,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D80" authorId="0" shapeId="0" xr:uid="{462043AC-24E8-4B01-BF3B-DBCE99D58342}">
+    <comment ref="D79" authorId="0" shapeId="0" xr:uid="{462043AC-24E8-4B01-BF3B-DBCE99D58342}">
       <text>
         <r>
           <rPr>
@@ -116,7 +116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C82" authorId="0" shapeId="0" xr:uid="{FB1C37D4-72C2-4D9F-A3A1-BE7E0FCFA979}">
+    <comment ref="C81" authorId="0" shapeId="0" xr:uid="{FB1C37D4-72C2-4D9F-A3A1-BE7E0FCFA979}">
       <text>
         <r>
           <rPr>
@@ -128,7 +128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D102" authorId="0" shapeId="0" xr:uid="{B95DBADC-5274-4970-B2EF-BA6EDE495B32}">
+    <comment ref="D101" authorId="0" shapeId="0" xr:uid="{B95DBADC-5274-4970-B2EF-BA6EDE495B32}">
       <text>
         <r>
           <rPr>
@@ -140,7 +140,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D110" authorId="0" shapeId="0" xr:uid="{3D1FECAA-E9AC-469D-968C-B08407A7E555}">
+    <comment ref="D109" authorId="0" shapeId="0" xr:uid="{3D1FECAA-E9AC-469D-968C-B08407A7E555}">
       <text>
         <r>
           <rPr>
@@ -152,7 +152,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D127" authorId="0" shapeId="0" xr:uid="{652EA41B-5E8F-4E35-965E-DC62524B30E4}">
+    <comment ref="D126" authorId="0" shapeId="0" xr:uid="{652EA41B-5E8F-4E35-965E-DC62524B30E4}">
       <text>
         <r>
           <rPr>
@@ -164,7 +164,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D132" authorId="0" shapeId="0" xr:uid="{EB3699E2-FEF4-456B-8D80-19A0E1F73915}">
+    <comment ref="D131" authorId="0" shapeId="0" xr:uid="{EB3699E2-FEF4-456B-8D80-19A0E1F73915}">
       <text>
         <r>
           <rPr>
@@ -177,7 +177,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E135" authorId="0" shapeId="0" xr:uid="{248F1982-A68D-4075-B49E-DFE7A3EEE35C}">
+    <comment ref="E134" authorId="0" shapeId="0" xr:uid="{248F1982-A68D-4075-B49E-DFE7A3EEE35C}">
       <text>
         <r>
           <rPr>
@@ -190,7 +190,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D137" authorId="0" shapeId="0" xr:uid="{146CA70A-EBE9-449B-8DB8-250759CFD077}">
+    <comment ref="D136" authorId="0" shapeId="0" xr:uid="{146CA70A-EBE9-449B-8DB8-250759CFD077}">
       <text>
         <r>
           <rPr>
@@ -203,7 +203,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D154" authorId="0" shapeId="0" xr:uid="{F773B15B-9F7C-43C0-94D6-9AFFA8926436}">
+    <comment ref="D153" authorId="0" shapeId="0" xr:uid="{F773B15B-9F7C-43C0-94D6-9AFFA8926436}">
       <text>
         <r>
           <rPr>
@@ -215,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E171" authorId="0" shapeId="0" xr:uid="{EF3CCB78-BD13-4482-8109-9AB59DD642A1}">
+    <comment ref="E170" authorId="0" shapeId="0" xr:uid="{EF3CCB78-BD13-4482-8109-9AB59DD642A1}">
       <text>
         <r>
           <rPr>
@@ -227,7 +227,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C180" authorId="0" shapeId="0" xr:uid="{5BDAADBF-92C0-4462-823A-597F00B6DA8B}">
+    <comment ref="C179" authorId="0" shapeId="0" xr:uid="{5BDAADBF-92C0-4462-823A-597F00B6DA8B}">
       <text>
         <r>
           <rPr>
@@ -239,7 +239,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C184" authorId="0" shapeId="0" xr:uid="{7115E3C1-ADBA-429A-AB3C-37FAE8BAC9C7}">
+    <comment ref="C183" authorId="0" shapeId="0" xr:uid="{7115E3C1-ADBA-429A-AB3C-37FAE8BAC9C7}">
       <text>
         <r>
           <rPr>
@@ -251,7 +251,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E231" authorId="0" shapeId="0" xr:uid="{EEE70887-3507-410D-908B-63439A987A79}">
+    <comment ref="E230" authorId="0" shapeId="0" xr:uid="{EEE70887-3507-410D-908B-63439A987A79}">
       <text>
         <r>
           <rPr>
@@ -264,7 +264,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D294" authorId="0" shapeId="0" xr:uid="{66A4E9CF-C1FD-417D-8D92-41FDF2D33936}">
+    <comment ref="D293" authorId="0" shapeId="0" xr:uid="{66A4E9CF-C1FD-417D-8D92-41FDF2D33936}">
       <text>
         <r>
           <rPr>
@@ -276,7 +276,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D316" authorId="0" shapeId="0" xr:uid="{F8960E51-4F3B-4B2F-AE76-558F4A32BC38}">
+    <comment ref="D315" authorId="0" shapeId="0" xr:uid="{F8960E51-4F3B-4B2F-AE76-558F4A32BC38}">
       <text>
         <r>
           <rPr>
@@ -293,20 +293,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
   <si>
     <t>MUZAKKI + ZAKIYAH</t>
   </si>
   <si>
-    <t xml:space="preserve"> ZUBAIDAH  + SHOLEH  + SHOLIHAHSULIHA Rabu malam Kamis, </t>
-  </si>
-  <si>
-    <t>ROFI'AH Alm</t>
-  </si>
-  <si>
-    <t>MALIHAH Alm  + ABDULLAH ABBAS Alm</t>
-  </si>
-  <si>
     <t>M NUR CHOLIS + USWATUN HASANAH</t>
   </si>
   <si>
@@ -322,9 +313,6 @@
     <t>AZZA MAISHARANI KHOIRUNNISA'</t>
   </si>
   <si>
-    <t>AZZA ALMIRA LALITYA</t>
-  </si>
-  <si>
     <t>AZZA SYAKIRA HASNA</t>
   </si>
   <si>
@@ -349,12 +337,6 @@
     <t>MUHAMMAD FAKHRI HASYIM</t>
   </si>
   <si>
-    <t>TOHA Alm waktu kecil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DJAMALIAH Alm  + SHOLEH BAIDLOWIAlm </t>
-  </si>
-  <si>
     <t>A MACHLUS SADAT + MAS'ULAH SIKHA AFIAH</t>
   </si>
   <si>
@@ -370,12 +352,6 @@
     <t>AHMAD FAKHRY AKRAMUSADAT</t>
   </si>
   <si>
-    <t>ALEESHA RALINE SALSABILA SADAT Kamis,</t>
-  </si>
-  <si>
-    <t>A MUCHLIS RIZAT Ahad Pon,  + USWATUN HASANAH</t>
-  </si>
-  <si>
     <t>SALIMATUL MAKKIYAH + M NAUFAL ZUHDI</t>
   </si>
   <si>
@@ -442,9 +418,6 @@
     <t>ASIAH AROFAT</t>
   </si>
   <si>
-    <t>MAZIDATUL FAIQOH Kamis Wage, + KHOTIB</t>
-  </si>
-  <si>
     <t>M ZAHID</t>
   </si>
   <si>
@@ -535,9 +508,6 @@
     <t>IBNU KHAIRUL AZZAM</t>
   </si>
   <si>
-    <t>FAHRUR ROZI Jumat,+ KHOIRIYAH</t>
-  </si>
-  <si>
     <t>FILDA QURROTU AINI + M NUR KHOZIN</t>
   </si>
   <si>
@@ -550,15 +520,6 @@
     <t>CHAURA ELMATLUBAH LUTFIAH</t>
   </si>
   <si>
-    <t>FAHRUR ROZI Jumat, + MAS'UDAH Jumat,</t>
-  </si>
-  <si>
-    <t>HABIBAH Alm Jumat,</t>
-  </si>
-  <si>
-    <t>M ZAKARIYAH Senin Kliwon, + IZZA MUFLIKAH</t>
-  </si>
-  <si>
     <t>LATHIFAH SAFARAH FALIH + RICCY VINDY PUTRA PERMANA</t>
   </si>
   <si>
@@ -574,9 +535,6 @@
     <t>HANA ELZAHRAH</t>
   </si>
   <si>
-    <t>ISTIQOMAH Alm waktu kecil</t>
-  </si>
-  <si>
     <t>KHOTIB SHOLEH + SITI LATHIFATUS SUN'IYAH</t>
   </si>
   <si>
@@ -589,9 +547,6 @@
     <t>MUHAMMAD IBRAHIM CHALIM</t>
   </si>
   <si>
-    <t xml:space="preserve">AHMADANI MUHAMMAD KHALLAF+NUN FATHATUS SHIVA Kamis Pahing, </t>
-  </si>
-  <si>
     <t>KEN ALI AHMAD MULLA</t>
   </si>
   <si>
@@ -607,9 +562,6 @@
     <t xml:space="preserve"> SALMAH  + HASAN NOER </t>
   </si>
   <si>
-    <t xml:space="preserve">M ROZIQIN HASAN  Senin  + SITI ROSYIDAH Selasa </t>
-  </si>
-  <si>
     <t>MAIDATUL HUSNAH + KHOIRUR ROFIK YUDI ALAMSYAH</t>
   </si>
   <si>
@@ -667,9 +619,6 @@
     <t>ANNISA SALSABILA AHMAD</t>
   </si>
   <si>
-    <t>M RIDLO'I almKamis, + SITI MUDRIKAH</t>
-  </si>
-  <si>
     <t>MOH MACHRUS ALI + JAZILATUN NI'MAH ISTRI KE</t>
   </si>
   <si>
@@ -712,9 +661,6 @@
     <t>A RIFQI NAUFAL</t>
   </si>
   <si>
-    <t>A MADANI Jumat + UMMI KULSUM</t>
-  </si>
-  <si>
     <t>SITI MUZAYANAH + M AMBIYA'</t>
   </si>
   <si>
@@ -763,9 +709,6 @@
     <t>ISA HAIDAR YULIANSAH+TRIANA WULANDARI</t>
   </si>
   <si>
-    <t xml:space="preserve">MAS'UDAH HASAN + MUCHLISUL AMAL Sabtu, </t>
-  </si>
-  <si>
     <t>AHMAD SHODIQUL MASDUQ + ATIK WAHYUNI</t>
   </si>
   <si>
@@ -781,9 +724,6 @@
     <t>ANNISA MAULIDI SYAVIRA</t>
   </si>
   <si>
-    <t>MASFUFAH HASAN + M MUCHDLOR Rabu,</t>
-  </si>
-  <si>
     <t>M FARID SANTOSO + NOVI HARIANI PUSPITASARI</t>
   </si>
   <si>
@@ -829,9 +769,6 @@
     <t>ANNE SALMA</t>
   </si>
   <si>
-    <t>M USMAN HASAN Sabtu Pon, + NIKMATUL HASANAH</t>
-  </si>
-  <si>
     <t>FILDA NURIS SILVI</t>
   </si>
   <si>
@@ -841,27 +778,15 @@
     <t>RIFKA AMALIA IFADHA</t>
   </si>
   <si>
-    <t>UMAR HASAN + DEWI FATMA Alm</t>
-  </si>
-  <si>
     <t>MOH NASIR SAGAF</t>
   </si>
   <si>
-    <t xml:space="preserve">MOH FAISHOL FAQIH Kamis,  </t>
-  </si>
-  <si>
-    <t>M FAHAD</t>
-  </si>
-  <si>
     <t>UMAR HASAN + MASTURAH</t>
   </si>
   <si>
     <t xml:space="preserve">MASRUROH HASAN + M IMRON </t>
   </si>
   <si>
-    <t>MIHSAN Alm</t>
-  </si>
-  <si>
     <t>AMIN QUTBI+KATRIN LUMBAN TOBING</t>
   </si>
   <si>
@@ -889,15 +814,6 @@
     <t>RUQOYYAH</t>
   </si>
   <si>
-    <t xml:space="preserve">ABDUL HARIS  alm umur  bulan </t>
-  </si>
-  <si>
-    <t>QUDSIYAH  + DJAUHARI Jumat  + ALFIYAH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DJUWAIRIYAH Rabu,+MUHAMMAD AMIN Alm </t>
-  </si>
-  <si>
     <t>MUFLIHAH AMIN + MUKHLIS YAHYA</t>
   </si>
   <si>
@@ -916,9 +832,6 @@
     <t>SYAGIFA ALYAN FARUHA</t>
   </si>
   <si>
-    <t xml:space="preserve">MAWADDAH + ROQIB Senin Legi, </t>
-  </si>
-  <si>
     <t>MUYASSAROH</t>
   </si>
   <si>
@@ -973,9 +886,6 @@
     <t>MAJDI MUAYYAD</t>
   </si>
   <si>
-    <t>FITRIYAH + ABD MUQIT Ahad,</t>
-  </si>
-  <si>
     <t>M FATHULLOH</t>
   </si>
   <si>
@@ -1021,21 +931,12 @@
     <t>BADI'UZZAMAN MALFATIH AZMATKHAN</t>
   </si>
   <si>
-    <t>ROBI'AH ADAWIYAH Alm</t>
-  </si>
-  <si>
-    <t>SYAMSUDDIN DJAUHARI Selasa Pon, + NA'IMAH</t>
-  </si>
-  <si>
     <t>LU'AILI ADDINA + MIRZA FAILASUFI</t>
   </si>
   <si>
     <t>MUHAMMAD RASYID FACHRUDDIN</t>
   </si>
   <si>
-    <t>MIFTAHUL FARIHAH Ahad Pon, + RIZKI MUSTAFANI</t>
-  </si>
-  <si>
     <t>M ZUHDI FARIZ ALGHOZALI MACHFUD</t>
   </si>
   <si>
@@ -1072,9 +973,6 @@
     <t>MUHAMMAD AZAM ASHFIYAK</t>
   </si>
   <si>
-    <t xml:space="preserve">MUNIFAH Jumat Wage, + UBAIDILLAH UMAR Senin Wage,  </t>
-  </si>
-  <si>
     <t>FARAQLIT RAMDLAN + WI'AM MURAD</t>
   </si>
   <si>
@@ -1102,9 +1000,6 @@
     <t>MOHAMMAD ALWI HAKIM</t>
   </si>
   <si>
-    <t xml:space="preserve">BADRUT TAMAM Alm Mkh, </t>
-  </si>
-  <si>
     <t>M ASYIK DJAUHARI + NUR INDAH</t>
   </si>
   <si>
@@ -1132,9 +1027,6 @@
     <t>MOH IZZUL AUZAD</t>
   </si>
   <si>
-    <t xml:space="preserve">QIBTIYAH + SUADI Kamis Pahing, </t>
-  </si>
-  <si>
     <t>MIKYATUL ADIYAH + M SYIFA'UDDIN</t>
   </si>
   <si>
@@ -1168,15 +1060,9 @@
     <t>MUHAMMAD AHNAF SARFARAZ ZAYYAN</t>
   </si>
   <si>
-    <t>MUSTHOFA Alm + MAIDATUL JANNAH</t>
-  </si>
-  <si>
     <t>NUR FITROTUL KAMILA*</t>
   </si>
   <si>
-    <t>MARIYAH ULFA Senin Legi,  + ZAINUL MUROD</t>
-  </si>
-  <si>
     <t>WI'AM MURAD+ FARAQLIT RAMDLAN</t>
   </si>
   <si>
@@ -1255,29 +1141,125 @@
     <t>SABIQ ZAIN MAKARIM</t>
   </si>
   <si>
-    <t>Generasi 1</t>
-  </si>
-  <si>
-    <t>Generasi 2</t>
-  </si>
-  <si>
-    <t>Generasi 3</t>
-  </si>
-  <si>
-    <t>Generasi 4</t>
-  </si>
-  <si>
-    <t>Generasi 5</t>
-  </si>
-  <si>
-    <t>Generasi 6</t>
+    <t xml:space="preserve"> ZUBAIDAH  + SHOLEH  + SHOLIHAHSULIHA</t>
+  </si>
+  <si>
+    <t>ROFI'AH</t>
+  </si>
+  <si>
+    <t>MALIHAH + ABDULLAH ABBAS</t>
+  </si>
+  <si>
+    <t>AZZAIRA LALITYA</t>
+  </si>
+  <si>
+    <t>UMAR HASAN + DEWI FATMA</t>
+  </si>
+  <si>
+    <t>MIHSAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABDUL HARIS  umur  bulan </t>
+  </si>
+  <si>
+    <t>ROBI'AH ADAWIYAH</t>
+  </si>
+  <si>
+    <t>MUSTHOFA + MAIDATUL JANNAH</t>
+  </si>
+  <si>
+    <t>DJAMALIAH  + SHOLEH BAIDLOWIA</t>
+  </si>
+  <si>
+    <t>M F</t>
+  </si>
+  <si>
+    <t>A MADANI  + UMMI KULSUM</t>
+  </si>
+  <si>
+    <t>QUDSIYAH  + DJAUHARI   + ALFIYAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M ROZIQIN HASAN    + SITI ROSYIDAH  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALEESHA RALINE SALSABILA SADAT </t>
+  </si>
+  <si>
+    <t>A MUCHLIS RIZAT   + USWATUN HASANAH</t>
+  </si>
+  <si>
+    <t>MAZIDATUL FAIQOH   + KHOTIB</t>
+  </si>
+  <si>
+    <t>FAHRUR ROZI + KHOIRIYAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAHRUR ROZI  + MAS'UDAH </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HABIBAH </t>
+  </si>
+  <si>
+    <t>M ZAKARIYAH   + IZZA MUFLIKAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AHMADANI MUHAMMAD KHALLAF+NUN FATHATUS SHIVA   </t>
+  </si>
+  <si>
+    <t>M RIDLO'I + SITI MUDRIKAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAS'UDAH HASAN + MUCHLISUL AMAL  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MASFUFAH HASAN + M MUCHDLOR </t>
+  </si>
+  <si>
+    <t>M USMAN HASAN  + NIKMATUL HASANAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOH FAISHOL FAQIH   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJUWAIRIYAH +MUHAMMAD AMIN </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAWADDAH + ROQIB   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FITRIYAH + ABD MUQIT </t>
+  </si>
+  <si>
+    <t>SYAMSUDDIN DJAUHARI  + NA'IMAH</t>
+  </si>
+  <si>
+    <t>MIFTAHUL FARIHAH  + RIZKI MUSTAFANI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUNIFAH   + UBAIDILLAH UMAR    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BADRUT TAMAM Mkh </t>
+  </si>
+  <si>
+    <t xml:space="preserve">QIBTIYAH + SUADI   </t>
+  </si>
+  <si>
+    <t>MARIYAH ULFA    + ZAINUL MUROD</t>
+  </si>
+  <si>
+    <t>TOHA</t>
+  </si>
+  <si>
+    <t>ISTIQOMAH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1291,25 +1273,13 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE5E7EB"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1324,9 +1294,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1342,10 +1311,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1646,7 +1611,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C629E1E-B955-4A3C-B56E-5C952373FF63}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F362"/>
+  <dimension ref="A1:F361"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -1657,1629 +1622,1609 @@
     <col min="6" max="6" width="28.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E11" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E12" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E13" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D14" t="s">
+    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D17" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="18" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E19" t="s">
-        <v>17</v>
+      <c r="C19" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>18</v>
+        <v>291</v>
       </c>
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C21" t="s">
-        <v>19</v>
+      <c r="D21" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>20</v>
+      <c r="E22" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="23" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
-        <v>24</v>
+        <v>296</v>
       </c>
     </row>
     <row r="27" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E27" t="s">
-        <v>25</v>
+      <c r="D27" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="28" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
-        <v>26</v>
+      <c r="E28" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E29" t="s">
-        <v>27</v>
+      <c r="F29" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="3:6" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="F31" t="s">
-        <v>29</v>
+      <c r="E31" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E32" t="s">
-        <v>30</v>
+      <c r="F32" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="33" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F34" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F35" t="s">
-        <v>33</v>
+      <c r="E35" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E36" t="s">
-        <v>34</v>
+      <c r="D36" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D37" t="s">
-        <v>35</v>
+      <c r="E37" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E38" t="s">
-        <v>36</v>
+      <c r="F38" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="39" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F39" t="s">
-        <v>37</v>
+      <c r="E39" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E40" t="s">
-        <v>38</v>
+      <c r="D40" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D42" t="s">
-        <v>40</v>
+      <c r="E42" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E43" t="s">
-        <v>41</v>
+      <c r="D43" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D44" t="s">
-        <v>42</v>
+      <c r="E44" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="47" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="48" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="49" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E50" t="s">
-        <v>48</v>
+      <c r="D50" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="51" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D51" t="s">
-        <v>49</v>
+      <c r="E51" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E53" t="s">
-        <v>51</v>
+      <c r="D53" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="55" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D55" t="s">
-        <v>53</v>
+      <c r="E55" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="56" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="57" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E57" t="s">
-        <v>55</v>
+      <c r="D57" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="58" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D58" t="s">
-        <v>56</v>
+      <c r="C58" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C59" t="s">
-        <v>57</v>
+      <c r="D59" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D60" t="s">
-        <v>58</v>
+      <c r="E60" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="61" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="62" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="63" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="64" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E64" t="s">
-        <v>62</v>
+      <c r="D64" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="65" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D65" t="s">
-        <v>63</v>
+      <c r="E65" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="66" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="67" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="68" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="69" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E69" t="s">
-        <v>67</v>
+      <c r="D69" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="70" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D70" t="s">
-        <v>68</v>
+      <c r="C70" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="71" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C71" t="s">
-        <v>69</v>
+      <c r="D71" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="72" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D72" t="s">
-        <v>70</v>
+      <c r="E72" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="73" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="74" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="75" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E75" t="s">
-        <v>73</v>
+      <c r="D75" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="76" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D76" t="s">
-        <v>74</v>
+      <c r="E76" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="77" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="78" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="79" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E79" t="s">
-        <v>77</v>
+      <c r="D79" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="80" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D80" t="s">
-        <v>78</v>
+      <c r="E80" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="81" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E81" t="s">
-        <v>79</v>
+      <c r="C81" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="82" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C82" t="s">
-        <v>80</v>
+      <c r="D82" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="83" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="84" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D84" t="s">
-        <v>82</v>
+      <c r="E84" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="85" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E85" t="s">
-        <v>83</v>
+      <c r="D85" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D86" t="s">
-        <v>84</v>
+      <c r="C86" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="87" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>85</v>
+        <v>301</v>
       </c>
     </row>
     <row r="88" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
-        <v>86</v>
+        <v>302</v>
       </c>
     </row>
     <row r="89" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C89" t="s">
-        <v>87</v>
+      <c r="D89" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="90" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D90" t="s">
-        <v>88</v>
+      <c r="E90" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="91" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E91" t="s">
-        <v>89</v>
+      <c r="D91" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="92" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="93" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D93" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D94" t="s">
-        <v>92</v>
+      <c r="C94" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="95" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="96" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C96" t="s">
-        <v>94</v>
+      <c r="D96" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D97" t="s">
-        <v>95</v>
+      <c r="E97" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E98" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E99" t="s">
-        <v>97</v>
+      <c r="D99" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D100" t="s">
-        <v>98</v>
+      <c r="E100" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E101" t="s">
-        <v>99</v>
+      <c r="D101" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D104" t="s">
-        <v>102</v>
+      <c r="B104" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B105" t="s">
-        <v>103</v>
+      <c r="C105" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C106" t="s">
-        <v>104</v>
+      <c r="D106" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="107" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D107" t="s">
-        <v>105</v>
+      <c r="E107" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="109" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E109" t="s">
-        <v>107</v>
+      <c r="D109" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="110" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D110" t="s">
-        <v>108</v>
+      <c r="E110" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E112" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E113" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
     </row>
     <row r="114" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E114" t="s">
-        <v>112</v>
+      <c r="D114" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="115" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D115" t="s">
-        <v>113</v>
+      <c r="E115" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="116" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
     </row>
     <row r="117" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="118" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E118" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="119" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E119" t="s">
-        <v>117</v>
+      <c r="D119" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="120" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D120" t="s">
-        <v>118</v>
+      <c r="E120" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="121" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E121" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
     </row>
     <row r="122" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E122" t="s">
-        <v>120</v>
+      <c r="D122" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="123" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D123" t="s">
-        <v>121</v>
+      <c r="E123" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="124" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
     </row>
     <row r="125" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E125" t="s">
-        <v>123</v>
+      <c r="C125" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="126" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C126" t="s">
-        <v>124</v>
+      <c r="D126" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="127" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D127" t="s">
-        <v>125</v>
+      <c r="E127" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="128" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E128" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
     </row>
     <row r="129" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E129" t="s">
-        <v>127</v>
+      <c r="D129" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="130" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D130" t="s">
-        <v>128</v>
+      <c r="E130" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="131" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E131" t="s">
-        <v>129</v>
+      <c r="D131" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="132" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D132" t="s">
-        <v>130</v>
+      <c r="E132" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="133" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E133" t="s">
-        <v>131</v>
+      <c r="D133" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="134" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D134" t="s">
-        <v>132</v>
+      <c r="E134" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="135" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E135" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
     </row>
     <row r="136" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E136" t="s">
-        <v>134</v>
+      <c r="D136" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="137" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D137" t="s">
-        <v>135</v>
+      <c r="E137" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="138" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E138" t="s">
-        <v>136</v>
+      <c r="D138" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="139" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D139" t="s">
-        <v>137</v>
+      <c r="E139" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="140" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E140" t="s">
-        <v>138</v>
+      <c r="C140" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="141" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C141" t="s">
-        <v>139</v>
+      <c r="D141" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="142" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D142" t="s">
-        <v>140</v>
+      <c r="E142" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="143" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E143" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
     </row>
     <row r="144" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E144" t="s">
-        <v>142</v>
+      <c r="D144" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="145" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D145" t="s">
-        <v>143</v>
+      <c r="E145" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="146" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E146" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
     </row>
     <row r="147" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E147" t="s">
-        <v>145</v>
+      <c r="C147" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="148" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C148" t="s">
-        <v>146</v>
+      <c r="D148" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="149" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D149" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
     </row>
     <row r="150" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D150" t="s">
-        <v>148</v>
+      <c r="E150" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="151" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E151" t="s">
-        <v>149</v>
+      <c r="D151" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="152" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D152" t="s">
-        <v>150</v>
+      <c r="C152" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="153" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C153" t="s">
-        <v>151</v>
+      <c r="D153" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="154" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D154" t="s">
-        <v>152</v>
+      <c r="E154" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="155" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E155" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
     </row>
     <row r="156" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E156" t="s">
-        <v>154</v>
+      <c r="D156" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="157" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D157" t="s">
-        <v>155</v>
+      <c r="C157" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="158" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C158" t="s">
-        <v>156</v>
+      <c r="D158" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="159" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D159" t="s">
-        <v>157</v>
+      <c r="E159" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="160" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E160" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
     </row>
     <row r="161" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E161" t="s">
-        <v>159</v>
+      <c r="D161" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="162" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D162" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
     </row>
     <row r="163" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D163" t="s">
-        <v>161</v>
+      <c r="C163" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="164" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C164" t="s">
-        <v>162</v>
+      <c r="D164" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="165" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D165" t="s">
-        <v>163</v>
+      <c r="E165" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="166" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
     </row>
     <row r="167" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E167" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
     </row>
     <row r="168" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E168" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
     </row>
     <row r="169" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E169" t="s">
-        <v>167</v>
+      <c r="D169" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="170" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D170" t="s">
-        <v>168</v>
+      <c r="E170" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="171" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E171" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
     </row>
     <row r="172" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E172" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
     </row>
     <row r="173" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E173" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="174" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E174" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
     </row>
     <row r="175" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E175" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
     </row>
     <row r="176" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E176" t="s">
-        <v>174</v>
+      <c r="D176" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="177" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D177" t="s">
-        <v>175</v>
+      <c r="E177" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="178" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E178" t="s">
-        <v>176</v>
+      <c r="D178" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="179" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D179" t="s">
-        <v>177</v>
+      <c r="C179" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="180" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C180" t="s">
-        <v>178</v>
+      <c r="D180" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="181" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D181" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
     </row>
     <row r="182" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D182" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
     </row>
     <row r="183" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D183" t="s">
-        <v>181</v>
+      <c r="C183" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="184" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C184" t="s">
-        <v>182</v>
+      <c r="D184" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="185" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D185" t="s">
-        <v>183</v>
+        <v>308</v>
       </c>
     </row>
     <row r="186" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D186" t="s">
-        <v>184</v>
+        <v>292</v>
       </c>
     </row>
     <row r="187" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D187" t="s">
-        <v>185</v>
+      <c r="C187" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="188" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C188" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
     </row>
     <row r="189" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C189" t="s">
-        <v>187</v>
+      <c r="D189" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="190" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D190" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
     </row>
     <row r="191" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D191" t="s">
-        <v>189</v>
+      <c r="E191" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="192" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E192" t="s">
-        <v>190</v>
+      <c r="D192" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="193" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D193" t="s">
-        <v>191</v>
+      <c r="E193" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="194" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E194" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
     </row>
     <row r="195" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E195" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
     </row>
     <row r="196" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E196" t="s">
-        <v>194</v>
+      <c r="D196" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="197" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D197" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
     </row>
     <row r="198" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D198" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
     </row>
     <row r="199" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D199" t="s">
-        <v>197</v>
+      <c r="C199" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="200" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C200" t="s">
-        <v>198</v>
+      <c r="B200" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="201" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B201" t="s">
-        <v>199</v>
+      <c r="C201" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="202" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C202" t="s">
-        <v>200</v>
+      <c r="D202" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="203" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D203" t="s">
-        <v>201</v>
+      <c r="E203" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="204" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E204" t="s">
-        <v>202</v>
+      <c r="F204" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="205" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F205" t="s">
-        <v>203</v>
+        <v>176</v>
       </c>
     </row>
     <row r="206" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="F206" t="s">
-        <v>204</v>
+      <c r="E206" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="207" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E207" t="s">
-        <v>205</v>
+        <v>178</v>
       </c>
     </row>
     <row r="208" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E208" t="s">
-        <v>206</v>
+      <c r="D208" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="209" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D209" t="s">
-        <v>207</v>
+      <c r="E209" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="210" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E210" t="s">
-        <v>208</v>
+        <v>180</v>
       </c>
     </row>
     <row r="211" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E211" t="s">
-        <v>209</v>
+        <v>181</v>
       </c>
     </row>
     <row r="212" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E212" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
     </row>
     <row r="213" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E213" t="s">
-        <v>211</v>
+        <v>183</v>
       </c>
     </row>
     <row r="214" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E214" t="s">
-        <v>212</v>
+        <v>184</v>
       </c>
     </row>
     <row r="215" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E215" t="s">
-        <v>213</v>
+      <c r="D215" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="216" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D216" t="s">
-        <v>214</v>
+      <c r="E216" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="217" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E217" t="s">
-        <v>215</v>
+      <c r="F217" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="218" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F218" t="s">
-        <v>216</v>
+        <v>188</v>
       </c>
     </row>
     <row r="219" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F219" t="s">
-        <v>217</v>
+        <v>189</v>
       </c>
     </row>
     <row r="220" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F220" t="s">
-        <v>218</v>
+      <c r="E220" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="221" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="E221" t="s">
-        <v>219</v>
+      <c r="F221" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="222" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="F222" t="s">
-        <v>220</v>
+      <c r="E222" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="223" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E223" t="s">
-        <v>221</v>
+        <v>193</v>
       </c>
     </row>
     <row r="224" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E224" t="s">
-        <v>222</v>
+        <v>194</v>
       </c>
     </row>
     <row r="225" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E225" t="s">
-        <v>223</v>
+        <v>195</v>
       </c>
     </row>
     <row r="226" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E226" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
     </row>
     <row r="227" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E227" t="s">
-        <v>225</v>
+      <c r="D227" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="228" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D228" t="s">
-        <v>226</v>
+      <c r="E228" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="229" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E229" t="s">
-        <v>227</v>
+        <v>198</v>
       </c>
     </row>
     <row r="230" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E230" t="s">
-        <v>228</v>
+        <v>199</v>
       </c>
     </row>
     <row r="231" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E231" t="s">
-        <v>229</v>
+        <v>200</v>
       </c>
     </row>
     <row r="232" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E232" t="s">
-        <v>230</v>
+        <v>201</v>
       </c>
     </row>
     <row r="233" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E233" t="s">
-        <v>231</v>
+      <c r="D233" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="234" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D234" t="s">
-        <v>232</v>
+      <c r="E234" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="235" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E235" t="s">
-        <v>233</v>
+        <v>204</v>
       </c>
     </row>
     <row r="236" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E236" t="s">
-        <v>234</v>
+      <c r="D236" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="237" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D237" t="s">
-        <v>235</v>
+      <c r="E237" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="238" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E238" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
     </row>
     <row r="239" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="E239" t="s">
-        <v>237</v>
+      <c r="D239" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="240" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D240" t="s">
-        <v>238</v>
+      <c r="E240" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="241" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E241" t="s">
-        <v>239</v>
+        <v>210</v>
       </c>
     </row>
     <row r="242" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E242" t="s">
-        <v>240</v>
+        <v>211</v>
       </c>
     </row>
     <row r="243" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E243" t="s">
-        <v>241</v>
+      <c r="C243" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="244" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C244" t="s">
-        <v>242</v>
+        <v>312</v>
       </c>
     </row>
     <row r="245" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C245" t="s">
-        <v>243</v>
+      <c r="D245" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="246" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D246" t="s">
-        <v>244</v>
+      <c r="E246" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="247" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E247" t="s">
-        <v>245</v>
+      <c r="D247" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="248" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D248" t="s">
-        <v>246</v>
+      <c r="E248" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="249" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E249" t="s">
-        <v>247</v>
+        <v>215</v>
       </c>
     </row>
     <row r="250" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E250" t="s">
-        <v>248</v>
+        <v>216</v>
       </c>
     </row>
     <row r="251" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E251" t="s">
-        <v>249</v>
+      <c r="D251" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="252" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D252" t="s">
-        <v>250</v>
+      <c r="E252" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="253" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E253" t="s">
-        <v>251</v>
+      <c r="D253" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="254" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D254" t="s">
-        <v>252</v>
+      <c r="E254" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="255" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E255" t="s">
-        <v>253</v>
+        <v>221</v>
       </c>
     </row>
     <row r="256" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E256" t="s">
-        <v>254</v>
+      <c r="D256" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="257" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D257" t="s">
-        <v>255</v>
+      <c r="E257" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="258" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E258" t="s">
-        <v>256</v>
+        <v>224</v>
       </c>
     </row>
     <row r="259" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E259" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
     </row>
     <row r="260" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E260" t="s">
-        <v>258</v>
+      <c r="C260" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="261" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C261" t="s">
-        <v>259</v>
+      <c r="D261" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="262" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D262" t="s">
-        <v>260</v>
+      <c r="E262" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="263" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E263" t="s">
-        <v>261</v>
+        <v>228</v>
       </c>
     </row>
     <row r="264" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E264" t="s">
-        <v>262</v>
+        <v>229</v>
       </c>
     </row>
     <row r="265" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E265" t="s">
-        <v>263</v>
+        <v>230</v>
       </c>
     </row>
     <row r="266" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E266" t="s">
-        <v>264</v>
+      <c r="D266" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="267" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D267" t="s">
-        <v>265</v>
+      <c r="E267" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="268" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E268" t="s">
-        <v>266</v>
+        <v>233</v>
       </c>
     </row>
     <row r="269" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E269" t="s">
-        <v>267</v>
+        <v>234</v>
       </c>
     </row>
     <row r="270" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E270" t="s">
-        <v>268</v>
+      <c r="D270" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="271" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D271" t="s">
-        <v>269</v>
+      <c r="C271" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="272" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C272" t="s">
-        <v>270</v>
+      <c r="D272" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="273" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D273" t="s">
-        <v>271</v>
+      <c r="E273" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="274" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E274" t="s">
-        <v>272</v>
+        <v>238</v>
       </c>
     </row>
     <row r="275" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E275" t="s">
-        <v>273</v>
+        <v>239</v>
       </c>
     </row>
     <row r="276" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E276" t="s">
-        <v>274</v>
+      <c r="D276" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="277" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D277" t="s">
-        <v>275</v>
+      <c r="E277" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="278" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E278" t="s">
-        <v>276</v>
+      <c r="D278" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="279" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D279" t="s">
-        <v>277</v>
+        <v>243</v>
       </c>
     </row>
     <row r="280" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D280" t="s">
-        <v>278</v>
+      <c r="C280" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="281" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C281" t="s">
-        <v>279</v>
+      <c r="D281" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="282" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D282" t="s">
-        <v>280</v>
+      <c r="E282" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="283" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E283" t="s">
-        <v>281</v>
+        <v>246</v>
       </c>
     </row>
     <row r="284" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E284" t="s">
-        <v>282</v>
+        <v>247</v>
       </c>
     </row>
     <row r="285" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E285" t="s">
-        <v>283</v>
+      <c r="D285" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="286" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D286" t="s">
-        <v>284</v>
+      <c r="E286" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="287" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E287" t="s">
-        <v>285</v>
+        <v>250</v>
       </c>
     </row>
     <row r="288" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E288" t="s">
-        <v>286</v>
+        <v>251</v>
       </c>
     </row>
     <row r="289" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E289" t="s">
-        <v>287</v>
+      <c r="D289" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="290" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D290" t="s">
-        <v>288</v>
+        <v>253</v>
       </c>
     </row>
     <row r="291" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D291" t="s">
-        <v>289</v>
+      <c r="E291" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="292" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E292" t="s">
+      <c r="C292" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="293" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C293" t="s">
-        <v>291</v>
+      <c r="D293" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="294" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D294" t="s">
-        <v>292</v>
+      <c r="C294" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="295" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C295" t="s">
-        <v>293</v>
+      <c r="D295" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="296" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D296" t="s">
-        <v>294</v>
+      <c r="E296" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="297" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E297" t="s">
-        <v>295</v>
+        <v>258</v>
       </c>
     </row>
     <row r="298" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E298" t="s">
-        <v>296</v>
+        <v>259</v>
       </c>
     </row>
     <row r="299" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E299" t="s">
-        <v>297</v>
+      <c r="D299" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="300" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D300" t="s">
-        <v>298</v>
+      <c r="E300" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="301" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E301" t="s">
-        <v>299</v>
+        <v>262</v>
       </c>
     </row>
     <row r="302" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E302" t="s">
-        <v>300</v>
+        <v>263</v>
       </c>
     </row>
     <row r="303" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E303" t="s">
-        <v>301</v>
+      <c r="D303" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="304" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D304" t="s">
-        <v>302</v>
+      <c r="E304" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="305" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E305" t="s">
-        <v>303</v>
+        <v>266</v>
       </c>
     </row>
     <row r="306" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E306" t="s">
-        <v>304</v>
+        <v>267</v>
       </c>
     </row>
     <row r="307" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E307" t="s">
-        <v>305</v>
+        <v>268</v>
       </c>
     </row>
     <row r="308" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E308" t="s">
-        <v>306</v>
+        <v>269</v>
       </c>
     </row>
     <row r="309" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E309" t="s">
-        <v>307</v>
+      <c r="D309" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="310" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D310" t="s">
-        <v>308</v>
+      <c r="E310" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="311" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E311" t="s">
-        <v>309</v>
+        <v>272</v>
       </c>
     </row>
     <row r="312" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E312" t="s">
-        <v>310</v>
+        <v>273</v>
       </c>
     </row>
     <row r="313" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E313" t="s">
-        <v>311</v>
+      <c r="D313" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="314" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D314" t="s">
-        <v>312</v>
+      <c r="C314" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="315" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C315" t="s">
-        <v>313</v>
+      <c r="D315" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="316" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D316" t="s">
-        <v>314</v>
+      <c r="C316" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="317" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C317" t="s">
-        <v>315</v>
+        <v>278</v>
       </c>
     </row>
     <row r="318" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C318" t="s">
-        <v>316</v>
+      <c r="D318" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="319" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D319" t="s">
-        <v>317</v>
+        <v>280</v>
       </c>
     </row>
     <row r="320" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D320" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="321" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D321" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="362" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F362">
-        <f>COUNTA(F2:F361)</f>
+        <v>281</v>
+      </c>
+    </row>
+    <row r="361" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F361">
+        <f>COUNTA(F1:F360)</f>
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement live search functionality for family members with AJAX support
</commit_message>
<xml_diff>
--- a/bani muzakki 2.xlsx
+++ b/bani muzakki 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4dd770f5288dd514/Documents/GitHub/familyhood.my.id/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D12EDC8A-B394-43F1-91E2-CF16B48B558C}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9E8225F-FEF6-4455-8A28-7AFE388BC41C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB80F8E-BB6F-464C-9455-26EC13A679BF}"/>
   </bookViews>
@@ -293,7 +293,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="318">
   <si>
     <t>MUZAKKI + ZAKIYAH</t>
   </si>
@@ -307,9 +307,6 @@
     <t>NASYWA AZZAHRO</t>
   </si>
   <si>
-    <t>AHMAD ZAKY +  YUYUN DWI WAHYUNI</t>
-  </si>
-  <si>
     <t>AZZA MAISHARANI KHOIRUNNISA'</t>
   </si>
   <si>
@@ -328,9 +325,6 @@
     <t>AISYAH NAILA SABRINA</t>
   </si>
   <si>
-    <t>FAUZAN FR +  AINI ZAHIDAH</t>
-  </si>
-  <si>
     <t>JANEETA EMIRA SHABRIYA</t>
   </si>
   <si>
@@ -391,9 +385,6 @@
     <t>MASLUH ANI AMIROH + TRI SUSANTO</t>
   </si>
   <si>
-    <t>MUKHLAS ARAFAT  + FARIDA S</t>
-  </si>
-  <si>
     <t>QONITA AROFAT</t>
   </si>
   <si>
@@ -427,18 +418,12 @@
     <t>MAZIDATUL FAIQOH + SEMIL SANTOSO</t>
   </si>
   <si>
-    <t>ANISATUS SHOBIHAH  + MUHAMMAD YUNANDI</t>
-  </si>
-  <si>
     <t>VINA NIHLATUR RAJWA</t>
   </si>
   <si>
     <t>ARINA HILYA EL HUSNA</t>
   </si>
   <si>
-    <t>RATU HUMAIRO  + LUTFI AFANDI</t>
-  </si>
-  <si>
     <t>SYAFIUDDIN + SITI ZUMAROH</t>
   </si>
   <si>
@@ -559,9 +544,6 @@
     <t>GHAZI BI LATHAIFILLAH ELKHOTIB</t>
   </si>
   <si>
-    <t xml:space="preserve"> SALMAH  + HASAN NOER </t>
-  </si>
-  <si>
     <t>MAIDATUL HUSNAH + KHOIRUR ROFIK YUDI ALAMSYAH</t>
   </si>
   <si>
@@ -739,9 +721,6 @@
     <t>ABDULLAH HANIF</t>
   </si>
   <si>
-    <t>VIVIEN FARIDAH +  M YASIN</t>
-  </si>
-  <si>
     <t xml:space="preserve">SILATUL FARHAH RIHADATUL AISY ASFA* + </t>
   </si>
   <si>
@@ -1060,9 +1039,6 @@
     <t>MUHAMMAD AHNAF SARFARAZ ZAYYAN</t>
   </si>
   <si>
-    <t>NUR FITROTUL KAMILA*</t>
-  </si>
-  <si>
     <t>WI'AM MURAD+ FARAQLIT RAMDLAN</t>
   </si>
   <si>
@@ -1123,9 +1099,6 @@
     <t>DAMANHURI + NUR MASLAHAH</t>
   </si>
   <si>
-    <t>JINDAN AHMAD ASRORI*</t>
-  </si>
-  <si>
     <t>FADHILAH</t>
   </si>
   <si>
@@ -1141,9 +1114,6 @@
     <t>SABIQ ZAIN MAKARIM</t>
   </si>
   <si>
-    <t xml:space="preserve"> ZUBAIDAH  + SHOLEH  + SHOLIHAHSULIHA</t>
-  </si>
-  <si>
     <t>ROFI'AH</t>
   </si>
   <si>
@@ -1159,100 +1129,124 @@
     <t>MIHSAN</t>
   </si>
   <si>
-    <t xml:space="preserve">ABDUL HARIS  umur  bulan </t>
-  </si>
-  <si>
     <t>ROBI'AH ADAWIYAH</t>
   </si>
   <si>
     <t>MUSTHOFA + MAIDATUL JANNAH</t>
   </si>
   <si>
-    <t>DJAMALIAH  + SHOLEH BAIDLOWIA</t>
-  </si>
-  <si>
     <t>M F</t>
   </si>
   <si>
-    <t>A MADANI  + UMMI KULSUM</t>
-  </si>
-  <si>
-    <t>QUDSIYAH  + DJAUHARI   + ALFIYAH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M ROZIQIN HASAN    + SITI ROSYIDAH  </t>
-  </si>
-  <si>
     <t xml:space="preserve">ALEESHA RALINE SALSABILA SADAT </t>
   </si>
   <si>
-    <t>A MUCHLIS RIZAT   + USWATUN HASANAH</t>
-  </si>
-  <si>
-    <t>MAZIDATUL FAIQOH   + KHOTIB</t>
-  </si>
-  <si>
     <t>FAHRUR ROZI + KHOIRIYAH</t>
   </si>
   <si>
-    <t xml:space="preserve">FAHRUR ROZI  + MAS'UDAH </t>
-  </si>
-  <si>
     <t xml:space="preserve">HABIBAH </t>
   </si>
   <si>
-    <t>M ZAKARIYAH   + IZZA MUFLIKAH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AHMADANI MUHAMMAD KHALLAF+NUN FATHATUS SHIVA   </t>
-  </si>
-  <si>
     <t>M RIDLO'I + SITI MUDRIKAH</t>
   </si>
   <si>
-    <t xml:space="preserve">MAS'UDAH HASAN + MUCHLISUL AMAL  </t>
-  </si>
-  <si>
     <t xml:space="preserve">MASFUFAH HASAN + M MUCHDLOR </t>
   </si>
   <si>
-    <t>M USMAN HASAN  + NIKMATUL HASANAH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOH FAISHOL FAQIH   </t>
-  </si>
-  <si>
     <t xml:space="preserve">DJUWAIRIYAH +MUHAMMAD AMIN </t>
   </si>
   <si>
-    <t xml:space="preserve">MAWADDAH + ROQIB   </t>
-  </si>
-  <si>
     <t xml:space="preserve">FITRIYAH + ABD MUQIT </t>
   </si>
   <si>
-    <t>SYAMSUDDIN DJAUHARI  + NA'IMAH</t>
-  </si>
-  <si>
-    <t>MIFTAHUL FARIHAH  + RIZKI MUSTAFANI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MUNIFAH   + UBAIDILLAH UMAR    </t>
-  </si>
-  <si>
     <t xml:space="preserve">BADRUT TAMAM Mkh </t>
   </si>
   <si>
-    <t xml:space="preserve">QIBTIYAH + SUADI   </t>
-  </si>
-  <si>
-    <t>MARIYAH ULFA    + ZAINUL MUROD</t>
-  </si>
-  <si>
     <t>TOHA</t>
   </si>
   <si>
     <t>ISTIQOMAH</t>
+  </si>
+  <si>
+    <t>ABDUL HARIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ZUBAIDAH + SHOLEH + SHOLIHAHSULIHA</t>
+  </si>
+  <si>
+    <t>AHMAD ZAKY + YUYUN DWI WAHYUNI</t>
+  </si>
+  <si>
+    <t>FAUZAN FR + AINI ZAHIDAH</t>
+  </si>
+  <si>
+    <t>DJAMALIAH + SHOLEH BAIDLOWIA</t>
+  </si>
+  <si>
+    <t>MUKHLAS ARAFAT + FARIDA S</t>
+  </si>
+  <si>
+    <t>ANISATUS SHOBIHAH + MUHAMMAD YUNANDI</t>
+  </si>
+  <si>
+    <t>RATU HUMAIRO + LUTFI AFANDI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAHRUR ROZI + MAS'UDAH </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SALMAH + HASAN NOER </t>
+  </si>
+  <si>
+    <t xml:space="preserve">M ROZIQIN HASAN + SITI ROSYIDAH </t>
+  </si>
+  <si>
+    <t>A MADANI + UMMI KULSUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAS'UDAH HASAN + MUCHLISUL AMAL </t>
+  </si>
+  <si>
+    <t>VIVIEN FARIDAH + M YASIN</t>
+  </si>
+  <si>
+    <t>M USMAN HASAN + NIKMATUL HASANAH</t>
+  </si>
+  <si>
+    <t>SYAMSUDDIN DJAUHARI + NA'IMAH</t>
+  </si>
+  <si>
+    <t>MIFTAHUL FARIHAH + RIZKI MUSTAFANI</t>
+  </si>
+  <si>
+    <t>A MUCHLIS RIZAT + USWATUN HASANAH</t>
+  </si>
+  <si>
+    <t>MAZIDATUL FAIQOH + KHOTIB</t>
+  </si>
+  <si>
+    <t>M ZAKARIYAH + IZZA MUFLIKAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AHMADANI MUHAMMAD KHALLAF+NUN FATHATUS SHIVA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOH FAISHOL FAQIH </t>
+  </si>
+  <si>
+    <t>QUDSIYAH + DJAUHARI + ALFIYAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAWADDAH + ROQIB </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MUNIFAH + UBAIDILLAH UMAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">QIBTIYAH + SUADI </t>
+  </si>
+  <si>
+    <t>MARIYAH ULFA + ZAINUL MUROD</t>
   </si>
 </sst>
 </file>
@@ -1311,6 +1305,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1629,17 +1627,17 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1659,1362 +1657,1362 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>4</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>11</v>
+        <v>294</v>
       </c>
     </row>
     <row r="17" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>318</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
     </row>
     <row r="27" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
-        <v>297</v>
+        <v>308</v>
       </c>
     </row>
     <row r="28" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E28" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="3:6" x14ac:dyDescent="0.25">
       <c r="F29" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="3:6" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E31" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="3:6" x14ac:dyDescent="0.25">
       <c r="F32" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F34" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E35" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E39" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="40" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
-        <v>32</v>
+        <v>296</v>
       </c>
     </row>
     <row r="42" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="46" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="49" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="50" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
-        <v>298</v>
+        <v>309</v>
       </c>
     </row>
     <row r="51" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
-        <v>44</v>
+        <v>297</v>
       </c>
     </row>
     <row r="55" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="56" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="57" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D57" t="s">
-        <v>47</v>
+        <v>298</v>
       </c>
     </row>
     <row r="58" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C58" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="59" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D59" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="60" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E60" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="63" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="64" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D64" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="65" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="67" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="69" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D69" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="70" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="71" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D71" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="72" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E72" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="73" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="74" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="75" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="76" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E76" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="77" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="78" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="79" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D79" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E80" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="81" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
     </row>
     <row r="82" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="83" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="84" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E84" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="85" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D85" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="86" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="87" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>301</v>
+        <v>283</v>
       </c>
     </row>
     <row r="88" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
     </row>
     <row r="89" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="90" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E90" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="91" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D91" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="92" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="93" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D93" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="94" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
-        <v>319</v>
+        <v>290</v>
       </c>
     </row>
     <row r="95" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="96" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D96" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E97" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E98" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E100" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
-        <v>88</v>
+        <v>300</v>
       </c>
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C105" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D106" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="107" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E107" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="109" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D109" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="110" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E110" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.25">
       <c r="E112" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E113" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="114" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D114" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="115" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E115" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="116" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="117" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="118" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E118" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="119" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D119" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="120" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E120" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="121" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E121" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="122" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D122" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="123" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E123" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="124" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="125" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C125" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
     </row>
     <row r="126" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D126" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="127" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E127" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E128" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="129" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D129" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="130" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E130" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="131" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D131" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="132" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E132" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="133" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D133" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="134" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E134" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="135" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E135" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="136" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D136" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="137" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E137" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="138" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D138" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="139" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E139" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="140" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
     </row>
     <row r="141" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D141" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="142" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E142" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="143" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E143" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="144" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D144" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="145" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E145" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="146" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E146" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="147" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C147" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="148" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D148" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="149" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D149" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="150" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E150" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="151" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D151" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="152" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C152" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="153" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D153" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="154" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E154" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="155" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E155" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="156" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D156" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="157" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C157" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="158" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D158" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="159" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E159" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="160" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E160" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="161" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D161" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="162" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D162" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="163" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C163" t="s">
-        <v>306</v>
+        <v>285</v>
       </c>
     </row>
     <row r="164" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D164" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="165" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E165" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="166" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="167" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E167" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="168" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E168" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="169" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D169" t="s">
-        <v>148</v>
+        <v>304</v>
       </c>
     </row>
     <row r="170" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E170" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="171" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E171" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="172" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E172" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="173" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E173" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="174" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E174" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="175" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E175" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="176" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D176" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="177" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E177" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
     </row>
     <row r="178" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D178" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="179" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C179" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="180" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D180" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="181" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D181" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="182" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D182" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="183" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C183" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
     </row>
     <row r="184" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D184" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="185" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D185" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="186" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D186" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
     </row>
     <row r="187" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C187" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="188" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C188" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="189" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D189" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
     </row>
     <row r="190" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D190" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="191" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E191" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="192" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D192" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="193" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E193" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="194" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E194" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="195" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E195" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="196" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D196" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="197" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D197" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="198" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D198" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="199" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C199" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="200" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B200" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
     </row>
     <row r="201" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C201" t="s">
-        <v>309</v>
+        <v>286</v>
       </c>
     </row>
     <row r="202" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D202" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="203" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E203" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="204" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F204" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="205" spans="2:6" x14ac:dyDescent="0.25">
       <c r="F205" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="206" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E206" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="207" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E207" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="208" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D208" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="209" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E209" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="210" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E210" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="211" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E211" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="212" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E212" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="213" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E213" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="214" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E214" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="215" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D215" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="216" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E216" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="217" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F217" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="218" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F218" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="219" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F219" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="220" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E220" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="221" spans="4:6" x14ac:dyDescent="0.25">
       <c r="F221" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="222" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E222" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="223" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E223" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="224" spans="4:6" x14ac:dyDescent="0.25">
       <c r="E224" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="225" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E225" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="226" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E226" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="227" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D227" t="s">
-        <v>311</v>
+        <v>287</v>
       </c>
     </row>
     <row r="228" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E228" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
     </row>
     <row r="229" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E229" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="230" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E230" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="231" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E231" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="232" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E232" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="233" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D233" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="234" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E234" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="235" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E235" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="236" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D236" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
     </row>
     <row r="237" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E237" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="238" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E238" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="239" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D239" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="240" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E240" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="241" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E241" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="242" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E242" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="243" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C243" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
     </row>
     <row r="244" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C244" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="245" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D245" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="246" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E246" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="247" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D247" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
     </row>
     <row r="248" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E248" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="249" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E249" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="250" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E250" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="251" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D251" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="252" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E252" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="253" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D253" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="254" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E254" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="255" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E255" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="256" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D256" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="257" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E257" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
     </row>
     <row r="258" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E258" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="259" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E259" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="260" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C260" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="261" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D261" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="262" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E262" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="263" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E263" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="264" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E264" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="265" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E265" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
     </row>
     <row r="266" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D266" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
     </row>
     <row r="267" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E267" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="268" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E268" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="269" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E269" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
     </row>
     <row r="270" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D270" t="s">
-        <v>315</v>
+        <v>288</v>
       </c>
     </row>
     <row r="271" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C271" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
     </row>
     <row r="272" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D272" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
     </row>
     <row r="273" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E273" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
     </row>
     <row r="274" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E274" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
     <row r="275" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E275" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="276" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D276" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="277" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E277" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
     </row>
     <row r="278" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D278" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
     </row>
     <row r="279" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D279" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="280" spans="3:5" x14ac:dyDescent="0.25">
@@ -3024,67 +3022,67 @@
     </row>
     <row r="281" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D281" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
     </row>
     <row r="282" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E282" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
     </row>
     <row r="283" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E283" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
     </row>
     <row r="284" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E284" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="285" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D285" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
     </row>
     <row r="286" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E286" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
     </row>
     <row r="287" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E287" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="288" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E288" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="289" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D289" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="290" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D290" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="291" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E291" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="292" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C292" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
     </row>
     <row r="293" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D293" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
     </row>
     <row r="294" spans="3:5" x14ac:dyDescent="0.25">
@@ -3094,132 +3092,132 @@
     </row>
     <row r="295" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D295" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
     </row>
     <row r="296" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E296" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
     </row>
     <row r="297" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E297" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="298" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E298" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
     </row>
     <row r="299" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D299" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="300" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E300" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
     </row>
     <row r="301" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E301" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="302" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E302" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
     </row>
     <row r="303" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D303" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
     </row>
     <row r="304" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E304" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
     </row>
     <row r="305" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E305" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="306" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E306" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="307" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E307" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="308" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E308" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
     </row>
     <row r="309" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D309" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
     </row>
     <row r="310" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E310" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
     </row>
     <row r="311" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E311" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="312" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E312" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
     </row>
     <row r="313" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D313" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
     </row>
     <row r="314" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C314" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
     </row>
     <row r="315" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D315" t="s">
-        <v>276</v>
+        <v>192</v>
       </c>
     </row>
     <row r="316" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C316" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
     </row>
     <row r="317" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C317" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
     </row>
     <row r="318" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D318" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
     </row>
     <row r="319" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D319" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
     </row>
     <row r="320" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D320" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="361" spans="6:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: close live search dropdown and clear input fields on content load
</commit_message>
<xml_diff>
--- a/bani muzakki 2.xlsx
+++ b/bani muzakki 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4dd770f5288dd514/Documents/GitHub/familyhood.my.id/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9E8225F-FEF6-4455-8A28-7AFE388BC41C}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{107DCD37-E142-49A6-A5C7-C5890FD142B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D35A4742-D70D-4464-B59E-3EC3BE51B38F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5BB80F8E-BB6F-464C-9455-26EC13A679BF}"/>
   </bookViews>
@@ -1135,9 +1135,6 @@
     <t>MUSTHOFA + MAIDATUL JANNAH</t>
   </si>
   <si>
-    <t>M F</t>
-  </si>
-  <si>
     <t xml:space="preserve">ALEESHA RALINE SALSABILA SADAT </t>
   </si>
   <si>
@@ -1247,6 +1244,9 @@
   </si>
   <si>
     <t>MARIYAH ULFA + ZAINUL MUROD</t>
+  </si>
+  <si>
+    <t>M FAHAD</t>
   </si>
 </sst>
 </file>
@@ -1609,7 +1609,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C629E1E-B955-4A3C-B56E-5C952373FF63}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F361"/>
+  <dimension ref="A1:F320"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -1627,7 +1627,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1657,7 +1657,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1697,7 +1697,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="17" spans="3:6" x14ac:dyDescent="0.25">
@@ -1712,12 +1712,12 @@
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
@@ -1747,12 +1747,12 @@
     </row>
     <row r="26" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="27" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="28" spans="3:6" x14ac:dyDescent="0.25">
@@ -1822,7 +1822,7 @@
     </row>
     <row r="41" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="42" spans="4:6" x14ac:dyDescent="0.25">
@@ -1867,7 +1867,7 @@
     </row>
     <row r="50" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="51" spans="3:5" x14ac:dyDescent="0.25">
@@ -1887,7 +1887,7 @@
     </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="55" spans="3:5" x14ac:dyDescent="0.25">
@@ -1902,7 +1902,7 @@
     </row>
     <row r="57" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D57" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="58" spans="3:5" x14ac:dyDescent="0.25">
@@ -2022,7 +2022,7 @@
     </row>
     <row r="81" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="82" spans="3:5" x14ac:dyDescent="0.25">
@@ -2047,17 +2047,17 @@
     </row>
     <row r="86" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C86" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="87" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C87" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="88" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C88" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="89" spans="3:5" x14ac:dyDescent="0.25">
@@ -2087,7 +2087,7 @@
     </row>
     <row r="94" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C94" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="95" spans="3:5" x14ac:dyDescent="0.25">
@@ -2112,7 +2112,7 @@
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.25">
@@ -2137,12 +2137,12 @@
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C105" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.25">
@@ -2242,7 +2242,7 @@
     </row>
     <row r="125" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C125" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="126" spans="3:5" x14ac:dyDescent="0.25">
@@ -2317,7 +2317,7 @@
     </row>
     <row r="140" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="141" spans="3:5" x14ac:dyDescent="0.25">
@@ -2402,7 +2402,7 @@
     </row>
     <row r="157" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C157" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="158" spans="3:5" x14ac:dyDescent="0.25">
@@ -2432,7 +2432,7 @@
     </row>
     <row r="163" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C163" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="164" spans="3:5" x14ac:dyDescent="0.25">
@@ -2462,7 +2462,7 @@
     </row>
     <row r="169" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D169" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="170" spans="3:5" x14ac:dyDescent="0.25">
@@ -2512,7 +2512,7 @@
     </row>
     <row r="179" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C179" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="180" spans="3:5" x14ac:dyDescent="0.25">
@@ -2542,12 +2542,12 @@
     </row>
     <row r="185" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D185" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="186" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D186" t="s">
-        <v>280</v>
+        <v>317</v>
       </c>
     </row>
     <row r="187" spans="3:5" x14ac:dyDescent="0.25">
@@ -2612,17 +2612,17 @@
     </row>
     <row r="199" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C199" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="200" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B200" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="201" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C201" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="202" spans="2:6" x14ac:dyDescent="0.25">
@@ -2657,7 +2657,7 @@
     </row>
     <row r="208" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D208" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="209" spans="4:6" x14ac:dyDescent="0.25">
@@ -2752,7 +2752,7 @@
     </row>
     <row r="227" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D227" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="228" spans="4:5" x14ac:dyDescent="0.25">
@@ -2837,7 +2837,7 @@
     </row>
     <row r="244" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C244" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="245" spans="3:5" x14ac:dyDescent="0.25">
@@ -2852,7 +2852,7 @@
     </row>
     <row r="247" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D247" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="248" spans="3:5" x14ac:dyDescent="0.25">
@@ -2917,7 +2917,7 @@
     </row>
     <row r="260" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C260" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="261" spans="3:5" x14ac:dyDescent="0.25">
@@ -2967,7 +2967,7 @@
     </row>
     <row r="270" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D270" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="271" spans="3:5" x14ac:dyDescent="0.25">
@@ -3017,7 +3017,7 @@
     </row>
     <row r="280" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C280" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="281" spans="3:5" x14ac:dyDescent="0.25">
@@ -3087,7 +3087,7 @@
     </row>
     <row r="294" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C294" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="295" spans="3:5" x14ac:dyDescent="0.25">
@@ -3218,12 +3218,6 @@
     <row r="320" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D320" t="s">
         <v>272</v>
-      </c>
-    </row>
-    <row r="361" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F361">
-        <f>COUNTA(F1:F360)</f>
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>